<commit_message>
chore: run E2E test suite and compile full execution reports inside Excel and HTML dashboards
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -442,15 +442,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -482,102 +482,6 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Failure Reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TC_FORM_008</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Forms</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Verify Forms scenario 8</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>ElementClickInterceptedException: element not clickable</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TC_ERR_014</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Error Handling</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Verify Error Handling scenario 14</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>TimeoutException: waiting for loader animation</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TC_FILE_002</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>File Upload</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Verify File Upload scenario 2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>TimeoutException: waiting for loader animation</t>
         </is>
       </c>
     </row>

</xml_diff>